<commit_message>
Elimination of parameter translations
Some parameters received facilitated options to make more friendly the way to introduce them into the parameters scripts, involving a "translating" process to convert the facilitated terms into variable and country codes. Now these translation processes were removed in order to simplify the scripts
</commit_message>
<xml_diff>
--- a/lista_paises.xlsx
+++ b/lista_paises.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26529"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAPFITOGEN3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hmpar\OneDrive\Documents\GitHub\Capfitogen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{397CC81E-2C4B-4E48-AF09-4546331148E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B014992F-F65E-45BA-9D8C-0918340A82DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1081,16 +1081,16 @@
     <t>ArabianPeninsula</t>
   </si>
   <si>
-    <t>Denomina</t>
-  </si>
-  <si>
     <t>sadc</t>
   </si>
   <si>
     <t>arabianpeninsula</t>
   </si>
   <si>
-    <t>Paises</t>
+    <t>Country code</t>
+  </si>
+  <si>
+    <t>Other descriptions</t>
   </si>
 </sst>
 </file>
@@ -1233,7 +1233,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1413,6 +1413,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -1574,8 +1580,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1938,11 +1945,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="B1" t="s">
         <v>356</v>
-      </c>
-      <c r="B1" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -3347,7 +3354,7 @@
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B177" t="s">
         <v>347</v>
@@ -3379,7 +3386,7 @@
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B181" t="s">
         <v>352</v>

</xml_diff>